<commit_message>
Version 1.1: Extending the USB port beyond the board outline and adding a version designation on the PCB
</commit_message>
<xml_diff>
--- a/hardware/docs/BOM.xlsx
+++ b/hardware/docs/BOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projekty\Battery power module\hardware\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60F7CF0D-4918-4F8E-B99D-088E2F845C7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A16E971-1635-4006-964E-A370BBC66B82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{A324B616-F4FA-4244-BF7B-25B903F1E59B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="41">
   <si>
     <t>Reference</t>
   </si>
@@ -111,15 +111,6 @@
   </si>
   <si>
     <t>https://www.usb.org/sites/default/files/documents/usb_type-c.zip</t>
-  </si>
-  <si>
-    <t>J2</t>
-  </si>
-  <si>
-    <t>Conn_01x02</t>
-  </si>
-  <si>
-    <t>Connector_JST:JST_PH_B2B-PH-K_1x02_P2.00mm_Vertical</t>
   </si>
   <si>
     <t>R1,R2</t>
@@ -192,7 +183,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -200,12 +191,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -579,7 +603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{126DE61E-F48A-4AC8-8FB3-26E51F197F66}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" bestFit="1" customWidth="1"/>
@@ -753,7 +777,7 @@
         <v>25</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" t="s">
         <v>26</v>
@@ -775,160 +799,147 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="A8" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B8">
-        <v>2</v>
-      </c>
-      <c r="C8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" t="s">
-        <v>10</v>
-      </c>
-      <c r="G8" t="s">
+      <c r="D8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="H8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>31</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E9" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" t="s">
-        <v>10</v>
-      </c>
-      <c r="G9" t="s">
-        <v>30</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11">
         <v>1</v>
       </c>
-      <c r="C10" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G10" t="s">
-        <v>30</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="C11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11">
-        <v>2</v>
-      </c>
-      <c r="C11" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G11" t="s">
-        <v>30</v>
-      </c>
-      <c r="H11" t="s">
-        <v>12</v>
-      </c>
-    </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="A12" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D12" t="s">
-        <v>10</v>
-      </c>
-      <c r="E12" t="s">
-        <v>10</v>
-      </c>
-      <c r="F12" t="s">
-        <v>10</v>
-      </c>
-      <c r="G12" t="s">
+      <c r="D12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H12" t="s">
-        <v>12</v>
+      <c r="H12" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>40</v>
-      </c>
-      <c r="B13">
-        <v>1</v>
-      </c>
-      <c r="C13" t="s">
-        <v>41</v>
-      </c>
-      <c r="D13" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13" t="s">
-        <v>10</v>
-      </c>
-      <c r="G13" t="s">
-        <v>42</v>
-      </c>
-      <c r="H13" t="s">
-        <v>43</v>
-      </c>
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="4"/>
+    </row>
+    <row r="19" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C19" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>